<commit_message>
progression bar added V1.0.3
</commit_message>
<xml_diff>
--- a/web_crawl/testing-data.xlsx
+++ b/web_crawl/testing-data.xlsx
@@ -1,120 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jimmy\Desktop\yapro\web_crawl\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C4F4B5-643D-4AF1-80BB-5A6D13A2711E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="testing-sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="testing-sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>單號</t>
-  </si>
-  <si>
-    <t>雅博單號</t>
-  </si>
-  <si>
-    <t>車牌號</t>
-  </si>
-  <si>
-    <t>收單日期</t>
-  </si>
-  <si>
-    <t>審核狀態</t>
-  </si>
-  <si>
-    <t>退稅方式</t>
-  </si>
-  <si>
-    <t>海關號碼</t>
-  </si>
-  <si>
-    <t>收件號碼</t>
-  </si>
-  <si>
-    <t>退/補件說明</t>
-  </si>
-  <si>
-    <t>審核完成日</t>
-  </si>
-  <si>
-    <t>退稅通知書製表日期</t>
-  </si>
-  <si>
-    <t>A001907</t>
-  </si>
-  <si>
-    <t>D-2025AB30-2000CC-23</t>
-  </si>
-  <si>
-    <t>CCN-3650</t>
-  </si>
-  <si>
-    <t>A001908</t>
-  </si>
-  <si>
-    <t>D-2025AB30-2000CC-24</t>
-  </si>
-  <si>
-    <t>CCA-8670</t>
-  </si>
-  <si>
-    <t>A001909</t>
-  </si>
-  <si>
-    <t>D-2025AB30-2000CC-25</t>
-  </si>
-  <si>
-    <t>CCA-8675</t>
-  </si>
-  <si>
-    <t>A001910</t>
-  </si>
-  <si>
-    <t>D-2025AB30-2000CC-26</t>
-  </si>
-  <si>
-    <t>CCA-8701</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <charset val="136"/>
+      <family val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="1"/>
-      <charset val="136"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -133,33 +54,92 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -479,135 +459,297 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col width="8.453125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="22.90625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.54296875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.08984375" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="8.81640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="14.08984375" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="11.453125" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="10.81640625" bestFit="1" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>10</v>
+    <row r="1" ht="43.5" customHeight="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>單號</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>雅博單號</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>車牌號</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>收單日期</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>審核狀態</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>退稅方式</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>海關號碼</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>收件號碼</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>退/補件說明</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>審核完成日</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>退稅通知書製表日期</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:11" s="3" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
+    <row r="2" ht="17" customFormat="1" customHeight="1" s="3">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>A001907</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-23</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CCN-3650</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
     </row>
-    <row r="3" spans="1:11" s="3" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3"/>
-      <c r="E3"/>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
-      <c r="J3"/>
-      <c r="K3"/>
+    <row r="3" ht="17" customFormat="1" customHeight="1" s="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>A001908</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-24</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CCA-8670</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
     </row>
-    <row r="4" spans="1:11" s="3" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4"/>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-      <c r="J4"/>
-      <c r="K4"/>
+    <row r="4" ht="17" customFormat="1" customHeight="1" s="3">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>A001909</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-25</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CCA-8675</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
     </row>
-    <row r="5" spans="1:11" s="3" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5"/>
-      <c r="I5"/>
-      <c r="J5"/>
-      <c r="K5"/>
+    <row r="5" ht="17" customFormat="1" customHeight="1" s="3">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>A001910</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-26</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>CCA-8701</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
     </row>
-    <row r="6" spans="1:11" s="3" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="2"/>
+    <row r="6" ht="17" customFormat="1" customHeight="1" s="3">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
V1.1.0 chinese version updated, copy function
</commit_message>
<xml_diff>
--- a/web_crawl/testing-data.xlsx
+++ b/web_crawl/testing-data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="testing-sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -575,38 +575,13 @@
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>審核完成</t>
+          <t>2026/01/16</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>
@@ -653,38 +628,13 @@
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>審核完成</t>
+          <t>2026/01/16</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>
@@ -731,38 +681,13 @@
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>審核完成</t>
+          <t>2026/01/16</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>
@@ -809,38 +734,13 @@
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>審核完成</t>
+          <t>2026/01/16</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>

</xml_diff>

<commit_message>
command line execution added
</commit_message>
<xml_diff>
--- a/web_crawl/testing-data.xlsx
+++ b/web_crawl/testing-data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="testing-sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -464,17 +464,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="8.453125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="22.90625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="9.54296875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.08984375" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="8.81640625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="14.08984375" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="11.453125" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="10.81640625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="8.44140625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="22.88671875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22.88671875" customWidth="1" min="3" max="3"/>
+    <col width="9.5546875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.109375" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="8.77734375" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="14.109375" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="11.44140625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="10.77734375" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="43.5" customHeight="1">
@@ -490,51 +491,56 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>車牌號</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>收單日期</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>審核狀態</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>退稅方式</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>海關號碼</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>收件號碼</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>退/補件說明</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>審核完成日</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>退稅通知書製表日期</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customFormat="1" customHeight="1" s="3">
+    <row r="2" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>A001907</t>
@@ -545,49 +551,54 @@
           <t>D-2025AB30-2000CC-23</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CCN-3650</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>2025/12/18</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>審核完成</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>直撥退車主</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>AB</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>2026/01/16</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="17" customFormat="1" customHeight="1" s="3">
+    <row r="3" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>A001908</t>
@@ -598,49 +609,54 @@
           <t>D-2025AB30-2000CC-24</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>CCA-8670</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>2025/12/18</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>審核完成</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>直撥退車主</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>AB</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
         <is>
           <t>2026/01/16</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="17" customFormat="1" customHeight="1" s="3">
+    <row r="4" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>A001909</t>
@@ -651,49 +667,54 @@
           <t>D-2025AB30-2000CC-25</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>CCA-8675</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>2025/12/18</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>審核完成</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>直撥退車主</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>AB</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
         <is>
           <t>2026/01/16</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customFormat="1" customHeight="1" s="3">
+    <row r="5" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>A001910</t>
@@ -704,52 +725,58 @@
           <t>D-2025AB30-2000CC-26</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>CCA-8701</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>2025/12/18</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>審核完成</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>直撥退車主</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>AB</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>AB20251218174</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
         <is>
           <t>2026/01/16</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026/02/02</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="17" customFormat="1" customHeight="1" s="3">
+    <row r="6" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A6" s="1" t="n"/>
       <c r="B6" s="1" t="n"/>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
output file option removed V1.3.0 updated
</commit_message>
<xml_diff>
--- a/web_crawl/testing-data.xlsx
+++ b/web_crawl/testing-data.xlsx
@@ -3,10 +3,11 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="testing-sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -561,42 +562,6 @@
           <t>CCN-3650</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>審核完成</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026/02/02</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A3" s="1" t="inlineStr">
@@ -619,42 +584,6 @@
           <t>CCA-8670</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>審核完成</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026/02/02</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A4" s="1" t="inlineStr">
@@ -677,42 +606,6 @@
           <t>CCA-8675</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>審核完成</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2026/02/02</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="16.95" customFormat="1" customHeight="1" s="3">
       <c r="A5" s="1" t="inlineStr">
@@ -733,42 +626,6 @@
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>CCA-8701</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2025/12/18</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>審核完成</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>直撥退車主</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>AB20251218174</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2026/01/16</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2026/02/02</t>
         </is>
       </c>
     </row>
@@ -782,4 +639,326 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" ht="43.2" customHeight="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>單號</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>雅博單號</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>車牌號</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>收單日期</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>審核狀態</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>退稅方式</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>海關號碼</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>收件號碼</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>退/補件說明</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>審核完成日</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>退稅通知書製表日期</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16.2" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>A001907</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-23</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>CCN-3650</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16.2" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>A001908</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-24</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>CCA-8670</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16.2" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>A001909</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-25</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>CCA-8675</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16.2" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>A001910</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>D-2025AB30-2000CC-26</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>CCA-8701</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2025/12/18</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>審核完成</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>直撥退車主</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AB20251218174</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026/01/16</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026/02/02</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16.2" customHeight="1">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>